<commit_message>
lots of updates to gene expression analysis
</commit_message>
<xml_diff>
--- a/gene_expression/readcounts_rawtrimmedaligned.xlsx
+++ b/gene_expression/readcounts_rawtrimmedaligned.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://miamiedu-my.sharepoint.com/personal/and128_miami_edu/Documents/GitHub/Ch2_temperaturevariability2023/gene_expression/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allysondemerlis/Documents/GitHub/temperaturevariabilityAcerPcli/gene_expression/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="8_{BD0676A9-DCF1-D347-8A65-AC01AF31CE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{883F1D9F-F73C-D645-9F8B-2623BF02327C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7827A797-B536-1C46-9D7A-92C11065A94D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20120" yWindow="500" windowWidth="19880" windowHeight="21020" activeTab="1" xr2:uid="{E30E7334-B642-5E4F-95D2-E511D28C5524}"/>
+    <workbookView xWindow="33600" yWindow="2740" windowWidth="28800" windowHeight="16280" activeTab="1" xr2:uid="{E30E7334-B642-5E4F-95D2-E511D28C5524}"/>
   </bookViews>
   <sheets>
     <sheet name="all samples" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
   <si>
     <t>Sample ID</t>
   </si>
@@ -400,6 +400,12 @@
   </si>
   <si>
     <t>Pcli alignment rate</t>
+  </si>
+  <si>
+    <t>SEM</t>
+  </si>
+  <si>
+    <t>count</t>
   </si>
 </sst>
 </file>
@@ -488,7 +494,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -519,6 +525,7 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,9 +545,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -578,7 +585,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -684,7 +691,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -826,7 +833,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4593,23 +4600,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{859AA9E9-E4AA-2B46-B9D7-BFBB7295C354}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>111</v>
       </c>
       <c r="C1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>113</v>
       </c>
@@ -4621,8 +4635,16 @@
         <f>STDEV('all samples'!B2:B49)</f>
         <v>2533563.1523973704</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D2">
+        <f>COUNT('all samples'!B2:B49)</f>
+        <v>48</v>
+      </c>
+      <c r="E2" s="12">
+        <f>C2/SQRT(D2)</f>
+        <v>365688.34201138467</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>114</v>
       </c>
@@ -4634,8 +4656,12 @@
         <f>STDEV('all samples'!G2:G49)</f>
         <v>1275745.4781924097</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <f>C3/SQRT(D2)</f>
+        <v>184137.99881295892</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>115</v>
       </c>
@@ -4647,8 +4673,12 @@
         <f>STDEV('all samples'!L2:L49)</f>
         <v>849685.86374670186</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <f>C4/SQRT(48)</f>
+        <v>122641.59054019451</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>116</v>
       </c>
@@ -4660,8 +4690,12 @@
         <f>STDEV('all samples'!M2:M49)</f>
         <v>3.8201409162710386E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <f>C5/SQRT(48)</f>
+        <v>5.5138984658784701E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>117</v>
       </c>
@@ -4673,8 +4707,16 @@
         <f>STDEV('all samples'!B50:B97)</f>
         <v>7019625.3202718673</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D6">
+        <f>COUNT('all samples'!B50:B97)</f>
+        <v>48</v>
+      </c>
+      <c r="E6">
+        <f>C6/SQRT(D6)</f>
+        <v>1013195.6420673189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>118</v>
       </c>
@@ -4686,8 +4728,12 @@
         <f>STDEV('all samples'!H50:H97)</f>
         <v>583464.39426871622</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <f>C7/SQRT(48)</f>
+        <v>84215.831273401316</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>119</v>
       </c>
@@ -4699,8 +4745,12 @@
         <f>STDEV('all samples'!N50:N97)</f>
         <v>537216.16221669572</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <f t="shared" ref="E8:E9" si="0">C8/SQRT(48)</f>
+        <v>77540.473967206737</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>120</v>
       </c>
@@ -4711,6 +4761,10 @@
       <c r="C9" s="10">
         <f>STDEV('all samples'!O50:O97)</f>
         <v>1.2328438625941124E-2</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>1.7794568398437221E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>